<commit_message>
Update template with ②白地 ODC formula fix and remove old ZIP
</commit_message>
<xml_diff>
--- a/保険金セグメント見積_v11_20260709.xlsx
+++ b/保険金セグメント見積_v11_20260709.xlsx
@@ -1965,17 +1965,20 @@
           <t>原価_国内（百万円）</t>
         </is>
       </c>
-      <c r="C46" s="23">
-        <f>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!C17*(1-(試算条件!C26+試算条件!C27))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34),$C$8*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C30)*(1-(試算条件!C26+試算条件!C27))*(1-試算条件!C20))</f>
-        <v/>
-      </c>
-      <c r="D46" s="23">
-        <f>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!D17*(1-(試算条件!D26+試算条件!D27))*(試算条件!D$33*試算条件!D$35+(1-試算条件!D$33)*試算条件!D$34),$C$8*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!D30)*(1-(試算条件!D26+試算条件!D27))*(1-試算条件!D20))</f>
-        <v/>
-      </c>
-      <c r="E46" s="23">
-        <f>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!E17*(1-(試算条件!E26+試算条件!E27))*(試算条件!E$33*試算条件!E$35+(1-試算条件!E$33)*試算条件!E$34),$C$8*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!E30)*(1-(試算条件!E26+試算条件!E27))*(1-試算条件!E20))</f>
-        <v/>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!C17*(1-(試算条件!C26+試算条件!C27))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*(1-試算条件!C20),$C$8*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C30)*(1-(試算条件!C26+試算条件!C27))*(1-試算条件!C20))</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!D17*(1-(試算条件!D26+試算条件!D27))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*(1-試算条件!D20),$C$8*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!C30)*(1-(試算条件!D26+試算条件!D27))*(1-試算条件!D20))</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!E17*(1-(試算条件!E26+試算条件!E27))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*(1-試算条件!E20),$C$8*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!C30)*(1-(試算条件!E26+試算条件!E27))*(1-試算条件!E20))</t>
+        </is>
       </c>
       <c r="F46" s="22">
         <f>SUM(C46:E46)</f>
@@ -1988,17 +1991,20 @@
           <t>原価_ODC（百万円）</t>
         </is>
       </c>
-      <c r="C47" s="23">
-        <f>IF($C$6="②COB白地",0,$C$8*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C30)*(1-(試算条件!C26+試算条件!C27))*試算条件!C20*試算条件!C21)</f>
-        <v/>
-      </c>
-      <c r="D47" s="23">
-        <f>IF($C$6="②COB白地",0,$C$8*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!D30)*(1-(試算条件!D26+試算条件!D27))*試算条件!D20*試算条件!D21)</f>
-        <v/>
-      </c>
-      <c r="E47" s="23">
-        <f>IF($C$6="②COB白地",0,$C$8*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!E30)*(1-(試算条件!E26+試算条件!E27))*試算条件!E20*試算条件!E21)</f>
-        <v/>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!C17*(1-(試算条件!C26+試算条件!C27))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*試算条件!C20*試算条件!C21,$C$8*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C30)*(1-(試算条件!C26+試算条件!C27))*試算条件!C20*試算条件!C21)</t>
+        </is>
+      </c>
+      <c r="D47" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!D17*(1-(試算条件!D26+試算条件!D27))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*試算条件!D20*試算条件!D21,$C$8*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!C30)*(1-(試算条件!D26+試算条件!D27))*試算条件!D20*試算条件!D21)</t>
+        </is>
+      </c>
+      <c r="E47" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$8*100*(1-試算条件!$C$10)*試算条件!E17*(1-(試算条件!E26+試算条件!E27))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*試算条件!E20*試算条件!E21,$C$8*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!C30)*(1-(試算条件!E26+試算条件!E27))*試算条件!E20*試算条件!E21)</t>
+        </is>
       </c>
       <c r="F47" s="22">
         <f>SUM(C47:E47)</f>
@@ -2207,17 +2213,20 @@
           <t>原価_国内（百万円）</t>
         </is>
       </c>
-      <c r="C58" s="23">
-        <f>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!C17*(1-(試算条件!C28+試算条件!C29))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34),$C$9*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C31)*(1-(試算条件!C28+試算条件!C29))*(1-試算条件!C20))</f>
-        <v/>
-      </c>
-      <c r="D58" s="23">
-        <f>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!D17*(1-(試算条件!D28+試算条件!D29))*(試算条件!D$33*試算条件!D$35+(1-試算条件!D$33)*試算条件!D$34),$C$9*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!D31)*(1-(試算条件!D28+試算条件!D29))*(1-試算条件!D20))</f>
-        <v/>
-      </c>
-      <c r="E58" s="23">
-        <f>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!E17*(1-(試算条件!E28+試算条件!E29))*(試算条件!E$33*試算条件!E$35+(1-試算条件!E$33)*試算条件!E$34),$C$9*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!E31)*(1-(試算条件!E28+試算条件!E29))*(1-試算条件!E20))</f>
-        <v/>
+      <c r="C58" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!C17*(1-(試算条件!C28+試算条件!C29))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*(1-試算条件!C20),$C$9*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C31)*(1-(試算条件!C28+試算条件!C29))*(1-試算条件!C20))</t>
+        </is>
+      </c>
+      <c r="D58" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!D17*(1-(試算条件!D28+試算条件!D29))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*(1-試算条件!D20),$C$9*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!C31)*(1-(試算条件!D28+試算条件!D29))*(1-試算条件!D20))</t>
+        </is>
+      </c>
+      <c r="E58" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!E17*(1-(試算条件!E28+試算条件!E29))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*(1-試算条件!E20),$C$9*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!C31)*(1-(試算条件!E28+試算条件!E29))*(1-試算条件!E20))</t>
+        </is>
       </c>
       <c r="F58" s="22">
         <f>SUM(C58:E58)</f>
@@ -2230,17 +2239,20 @@
           <t>原価_ODC（百万円）</t>
         </is>
       </c>
-      <c r="C59" s="23">
-        <f>IF($C$6="②COB白地",0,$C$9*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C31)*(1-(試算条件!C28+試算条件!C29))*試算条件!C20*試算条件!C21)</f>
-        <v/>
-      </c>
-      <c r="D59" s="23">
-        <f>IF($C$6="②COB白地",0,$C$9*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!D31)*(1-(試算条件!D28+試算条件!D29))*試算条件!D20*試算条件!D21)</f>
-        <v/>
-      </c>
-      <c r="E59" s="23">
-        <f>IF($C$6="②COB白地",0,$C$9*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!E31)*(1-(試算条件!E28+試算条件!E29))*試算条件!E20*試算条件!E21)</f>
-        <v/>
+      <c r="C59" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!C17*(1-(試算条件!C28+試算条件!C29))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*試算条件!C20*試算条件!C21,$C$9*100*(1-試算条件!$C$10)*試算条件!C17*(1-試算条件!C31)*(1-(試算条件!C28+試算条件!C29))*試算条件!C20*試算条件!C21)</t>
+        </is>
+      </c>
+      <c r="D59" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!D17*(1-(試算条件!D28+試算条件!D29))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*試算条件!D20*試算条件!D21,$C$9*100*(1-試算条件!$C$10)*試算条件!D17*(1-試算条件!C31)*(1-(試算条件!D28+試算条件!D29))*試算条件!D20*試算条件!D21)</t>
+        </is>
+      </c>
+      <c r="E59" s="23" t="inlineStr">
+        <is>
+          <t>IF($C$6="②COB白地",$C$9*100*(1-試算条件!$C$10)*試算条件!E17*(1-(試算条件!E28+試算条件!E29))*(試算条件!C$33*試算条件!C$35+(1-試算条件!C$33)*試算条件!C$34)*試算条件!E20*試算条件!E21,$C$9*100*(1-試算条件!$C$10)*試算条件!E17*(1-試算条件!C31)*(1-(試算条件!E28+試算条件!E29))*試算条件!E20*試算条件!E21)</t>
+        </is>
       </c>
       <c r="F59" s="22">
         <f>SUM(C59:E59)</f>

</xml_diff>